<commit_message>
maj du code front
</commit_message>
<xml_diff>
--- a/front/valy/src/assets/economie/economic_calendar_sections.xlsx
+++ b/front/valy/src/assets/economie/economic_calendar_sections.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="32">
   <si>
     <t>Time</t>
   </si>
@@ -37,160 +37,79 @@
     <t>Previous</t>
   </si>
   <si>
-    <t>17:00</t>
-  </si>
-  <si>
-    <t>16:45</t>
-  </si>
-  <si>
-    <t>17:30</t>
-  </si>
-  <si>
     <t>21:00</t>
   </si>
   <si>
-    <t>21:30</t>
-  </si>
-  <si>
-    <t>06:00</t>
-  </si>
-  <si>
-    <t>15:30</t>
-  </si>
-  <si>
-    <t>16:15</t>
-  </si>
-  <si>
-    <t>13:00</t>
+    <t>10:00</t>
+  </si>
+  <si>
+    <t>20:00</t>
   </si>
   <si>
     <t>USD</t>
   </si>
   <si>
-    <t>CAD</t>
-  </si>
-  <si>
-    <t>JPY</t>
-  </si>
-  <si>
-    <t>EUR</t>
-  </si>
-  <si>
-    <t>CB Consumer Confidence (Oct)</t>
-  </si>
-  <si>
-    <t>BoC Interest Rate Decision</t>
-  </si>
-  <si>
-    <t>New Home Sales (Sep)</t>
+    <t>GBP</t>
+  </si>
+  <si>
+    <t>10-Year Note Auction</t>
+  </si>
+  <si>
+    <t>GDP (QoQ) (Q3)</t>
+  </si>
+  <si>
+    <t>GDP (YoY) (Q3)</t>
+  </si>
+  <si>
+    <t>GDP (MoM) (Sep)</t>
   </si>
   <si>
     <t>Crude Oil Inventories</t>
   </si>
   <si>
-    <t>FOMC Statement</t>
-  </si>
-  <si>
-    <t>Fed Interest Rate Decision</t>
-  </si>
-  <si>
-    <t>FOMC Press Conference</t>
-  </si>
-  <si>
-    <t>BoJ Interest Rate Decision</t>
-  </si>
-  <si>
-    <t>GDP (QoQ) (Q3)</t>
-  </si>
-  <si>
-    <t>Deposit Facility Rate (Oct)</t>
-  </si>
-  <si>
-    <t>ECB Interest Rate Decision (Oct)</t>
-  </si>
-  <si>
-    <t>ECB Press Conference</t>
-  </si>
-  <si>
-    <t>CPI (YoY) (Oct)</t>
-  </si>
-  <si>
-    <t>Core PCE Price Index (YoY) (Sep)</t>
-  </si>
-  <si>
-    <t>Core PCE Price Index (MoM) (Sep)</t>
-  </si>
-  <si>
-    <t>Chicago PMI (Oct)</t>
-  </si>
-  <si>
-    <t>94.6</t>
-  </si>
-  <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>93.4</t>
-  </si>
-  <si>
-    <t>2.25%</t>
-  </si>
-  <si>
-    <t>710K</t>
-  </si>
-  <si>
-    <t>-0.400M</t>
-  </si>
-  <si>
-    <t>4.00%</t>
-  </si>
-  <si>
-    <t>0.50%</t>
-  </si>
-  <si>
-    <t>3.0%</t>
-  </si>
-  <si>
-    <t>2.00%</t>
-  </si>
-  <si>
-    <t>2.15%</t>
-  </si>
-  <si>
-    <t>2.1%</t>
+    <t>30-Year Bond Auction</t>
+  </si>
+  <si>
+    <t>4.074%</t>
+  </si>
+  <si>
+    <t>0.1%</t>
+  </si>
+  <si>
+    <t>1.3%</t>
+  </si>
+  <si>
+    <t>-0.1%</t>
+  </si>
+  <si>
+    <t>6.413M</t>
+  </si>
+  <si>
+    <t>4.694%</t>
   </si>
   <si>
     <t>0.2%</t>
   </si>
   <si>
-    <t>42.0</t>
-  </si>
-  <si>
-    <t>95.6</t>
-  </si>
-  <si>
-    <t>2.50%</t>
-  </si>
-  <si>
-    <t>800K</t>
-  </si>
-  <si>
-    <t>-0.961M</t>
-  </si>
-  <si>
-    <t>4.25%</t>
-  </si>
-  <si>
-    <t>3.8%</t>
-  </si>
-  <si>
-    <t>2.2%</t>
-  </si>
-  <si>
-    <t>2.9%</t>
-  </si>
-  <si>
-    <t>40.6</t>
+    <t>0.0%</t>
+  </si>
+  <si>
+    <t>1.000M</t>
+  </si>
+  <si>
+    <t>4.117%</t>
+  </si>
+  <si>
+    <t>0.3%</t>
+  </si>
+  <si>
+    <t>1.4%</t>
+  </si>
+  <si>
+    <t>5.202M</t>
+  </si>
+  <si>
+    <t>4.734%</t>
   </si>
 </sst>
 </file>
@@ -548,7 +467,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -576,7 +495,7 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2">
-        <f>== Tuesday, October 28, 2025 ===</f>
+        <f>== Wednesday, November 12, 2025 ===</f>
         <v>0</v>
       </c>
     </row>
@@ -585,24 +504,21 @@
         <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="D3" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="E3" t="s">
-        <v>36</v>
-      </c>
-      <c r="F3" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="G3" t="s">
-        <v>50</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5">
-        <f>== Wednesday, October 29, 2025 ===</f>
+        <f>== Thursday, November 13, 2025 ===</f>
         <v>0</v>
       </c>
     </row>
@@ -611,290 +527,96 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="D6" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="E6" t="s">
-        <v>37</v>
+        <v>19</v>
       </c>
       <c r="F6" t="s">
-        <v>39</v>
+        <v>24</v>
       </c>
       <c r="G6" t="s">
-        <v>51</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D7" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="E7" t="s">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="F7" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="G7" t="s">
-        <v>52</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D8" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="E8" t="s">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="F8" t="s">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="G8" t="s">
-        <v>53</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
         <v>10</v>
       </c>
-      <c r="B9" t="s">
+      <c r="D9" t="s">
         <v>16</v>
       </c>
-      <c r="D9" t="s">
-        <v>24</v>
-      </c>
       <c r="E9" t="s">
-        <v>37</v>
+        <v>22</v>
+      </c>
+      <c r="F9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G9" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" t="s">
         <v>10</v>
       </c>
-      <c r="B10" t="s">
-        <v>16</v>
-      </c>
       <c r="D10" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="E10" t="s">
-        <v>37</v>
-      </c>
-      <c r="F10" t="s">
-        <v>42</v>
+        <v>23</v>
       </c>
       <c r="G10" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7">
-      <c r="A11" t="s">
-        <v>11</v>
-      </c>
-      <c r="B11" t="s">
-        <v>16</v>
-      </c>
-      <c r="D11" t="s">
-        <v>26</v>
-      </c>
-      <c r="E11" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7">
-      <c r="A13">
-        <f>== Thursday, October 30, 2025 ===</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7">
-      <c r="A14" t="s">
-        <v>12</v>
-      </c>
-      <c r="B14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D14" t="s">
-        <v>27</v>
-      </c>
-      <c r="E14" t="s">
-        <v>37</v>
-      </c>
-      <c r="F14" t="s">
-        <v>43</v>
-      </c>
-      <c r="G14" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7">
-      <c r="A15" t="s">
-        <v>13</v>
-      </c>
-      <c r="B15" t="s">
-        <v>16</v>
-      </c>
-      <c r="D15" t="s">
-        <v>28</v>
-      </c>
-      <c r="E15" t="s">
-        <v>37</v>
-      </c>
-      <c r="F15" t="s">
-        <v>44</v>
-      </c>
-      <c r="G15" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7">
-      <c r="A16" t="s">
-        <v>14</v>
-      </c>
-      <c r="B16" t="s">
-        <v>19</v>
-      </c>
-      <c r="D16" t="s">
-        <v>29</v>
-      </c>
-      <c r="E16" t="s">
-        <v>37</v>
-      </c>
-      <c r="F16" t="s">
-        <v>45</v>
-      </c>
-      <c r="G16" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7">
-      <c r="A17" t="s">
-        <v>14</v>
-      </c>
-      <c r="B17" t="s">
-        <v>19</v>
-      </c>
-      <c r="D17" t="s">
-        <v>30</v>
-      </c>
-      <c r="E17" t="s">
-        <v>37</v>
-      </c>
-      <c r="F17" t="s">
-        <v>46</v>
-      </c>
-      <c r="G17" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7">
-      <c r="A18" t="s">
-        <v>8</v>
-      </c>
-      <c r="B18" t="s">
-        <v>19</v>
-      </c>
-      <c r="D18" t="s">
         <v>31</v>
-      </c>
-      <c r="E18" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7">
-      <c r="A20">
-        <f>== Friday, October 31, 2025 ===</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7">
-      <c r="A21" t="s">
-        <v>15</v>
-      </c>
-      <c r="B21" t="s">
-        <v>19</v>
-      </c>
-      <c r="D21" t="s">
-        <v>32</v>
-      </c>
-      <c r="E21" t="s">
-        <v>37</v>
-      </c>
-      <c r="F21" t="s">
-        <v>47</v>
-      </c>
-      <c r="G21" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7">
-      <c r="A22" t="s">
-        <v>13</v>
-      </c>
-      <c r="B22" t="s">
-        <v>16</v>
-      </c>
-      <c r="D22" t="s">
-        <v>33</v>
-      </c>
-      <c r="E22" t="s">
-        <v>37</v>
-      </c>
-      <c r="G22" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7">
-      <c r="A23" t="s">
-        <v>13</v>
-      </c>
-      <c r="B23" t="s">
-        <v>16</v>
-      </c>
-      <c r="D23" t="s">
-        <v>34</v>
-      </c>
-      <c r="E23" t="s">
-        <v>37</v>
-      </c>
-      <c r="F23" t="s">
-        <v>48</v>
-      </c>
-      <c r="G23" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7">
-      <c r="A24" t="s">
-        <v>8</v>
-      </c>
-      <c r="B24" t="s">
-        <v>16</v>
-      </c>
-      <c r="D24" t="s">
-        <v>35</v>
-      </c>
-      <c r="E24" t="s">
-        <v>37</v>
-      </c>
-      <c r="F24" t="s">
-        <v>49</v>
-      </c>
-      <c r="G24" t="s">
-        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>